<commit_message>
Updated Fixes For Reverse Grn Test Scenarios
Updated Fixes For Reverse Grn Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/PMF - Scenarios2.xlsx
+++ b/testdata/PMF - Scenarios2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1974" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2261" uniqueCount="155">
   <si>
     <t>Production Order - All Inside</t>
   </si>
@@ -348,6 +348,15 @@
     <t>6</t>
   </si>
   <si>
+    <t>99627</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>99637</t>
+  </si>
+  <si>
     <t>99711</t>
   </si>
   <si>
@@ -357,7 +366,22 @@
     <t>GWLD-IEC-FIFO-LOT-BATCH-10001(FG)</t>
   </si>
   <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>2600</t>
+  </si>
+  <si>
     <t>Material Request &amp; Material Issuance Voucher &amp; Completion After Consumption</t>
+  </si>
+  <si>
+    <t>Current Qty</t>
+  </si>
+  <si>
+    <t>99647</t>
+  </si>
+  <si>
+    <t>99708</t>
   </si>
   <si>
     <t>BOM-2627-0000804</t>
@@ -367,9 +391,6 @@
   </si>
   <si>
     <t>99774</t>
-  </si>
-  <si>
-    <t>3</t>
   </si>
   <si>
     <t>GWLD-FIFO-LOT-BATCH-10002(RM)</t>
@@ -424,6 +445,57 @@
   </si>
   <si>
     <t>99753</t>
+  </si>
+  <si>
+    <t>99695</t>
+  </si>
+  <si>
+    <t>99624</t>
+  </si>
+  <si>
+    <t>99634</t>
+  </si>
+  <si>
+    <t>99618</t>
+  </si>
+  <si>
+    <t>99628</t>
+  </si>
+  <si>
+    <t>99615</t>
+  </si>
+  <si>
+    <t>99625</t>
+  </si>
+  <si>
+    <t>99612</t>
+  </si>
+  <si>
+    <t>99622</t>
+  </si>
+  <si>
+    <t>99609</t>
+  </si>
+  <si>
+    <t>99619</t>
+  </si>
+  <si>
+    <t>99606</t>
+  </si>
+  <si>
+    <t>99616</t>
+  </si>
+  <si>
+    <t>99603</t>
+  </si>
+  <si>
+    <t>99613</t>
+  </si>
+  <si>
+    <t>99600</t>
+  </si>
+  <si>
+    <t>99610</t>
   </si>
 </sst>
 </file>
@@ -1221,7 +1293,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1814,23 +1886,23 @@
   <dimension ref="A1:XEQ69"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="12.1428571428571" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.8190476190476" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.2761904761905" style="1" customWidth="1"/>
-    <col min="4" max="5" width="34.4571428571429" style="1" customWidth="1"/>
-    <col min="6" max="9" width="34.2761904761905" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15.3619047619048" style="1" customWidth="1"/>
-    <col min="11" max="11" width="34.2761904761905" style="1" customWidth="1"/>
-    <col min="12" max="12" width="14.3619047619048" style="1" customWidth="1"/>
-    <col min="13" max="13" width="16.1809523809524" style="1" customWidth="1"/>
-    <col min="14" max="14" width="19.3619047619048" style="1" customWidth="1"/>
-    <col min="15" max="15" width="19.6380952380952" style="1" customWidth="1"/>
-    <col min="16" max="16" width="15.9047619047619" style="1" customWidth="1"/>
-    <col min="17" max="17" width="21.1809523809524" style="1" customWidth="1"/>
-    <col min="18" max="18" width="16.2857142857143" style="1" customWidth="1"/>
-    <col min="19" max="21" width="19.6380952380952" style="1" customWidth="1"/>
-    <col min="22" max="16371" width="9.13333333333333" style="1"/>
-    <col min="16372" max="16384" width="9" style="2"/>
+    <col min="1" max="1" customWidth="true" style="1" width="12.1428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="11.8190476190476"/>
+    <col min="3" max="3" customWidth="true" style="1" width="17.2761904761905"/>
+    <col min="4" max="5" customWidth="true" style="1" width="34.4571428571429"/>
+    <col min="6" max="9" customWidth="true" style="1" width="34.2761904761905"/>
+    <col min="10" max="10" customWidth="true" style="1" width="15.3619047619048"/>
+    <col min="11" max="11" customWidth="true" style="1" width="34.2761904761905"/>
+    <col min="12" max="12" customWidth="true" style="1" width="14.3619047619048"/>
+    <col min="13" max="13" customWidth="true" style="1" width="16.1809523809524"/>
+    <col min="14" max="14" customWidth="true" style="1" width="19.3619047619048"/>
+    <col min="15" max="15" customWidth="true" style="1" width="19.6380952380952"/>
+    <col min="16" max="16" customWidth="true" style="1" width="15.9047619047619"/>
+    <col min="17" max="17" customWidth="true" style="1" width="21.1809523809524"/>
+    <col min="18" max="18" customWidth="true" style="1" width="16.2857142857143"/>
+    <col min="19" max="21" customWidth="true" style="1" width="19.6380952380952"/>
+    <col min="22" max="16371" style="1" width="9.13333333333333"/>
+    <col min="16372" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33 16370:16371">
@@ -4915,23 +4987,23 @@
   <dimension ref="A1:XEQ69"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="12.1428571428571" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.8190476190476" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.2761904761905" style="1" customWidth="1"/>
-    <col min="4" max="5" width="34.4571428571429" style="1" customWidth="1"/>
-    <col min="6" max="9" width="34.2761904761905" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15.3619047619048" style="1" customWidth="1"/>
-    <col min="11" max="11" width="34.2761904761905" style="1" customWidth="1"/>
-    <col min="12" max="12" width="14.3619047619048" style="1" customWidth="1"/>
-    <col min="13" max="13" width="16.1809523809524" style="1" customWidth="1"/>
-    <col min="14" max="14" width="19.3619047619048" style="1" customWidth="1"/>
-    <col min="15" max="15" width="19.6380952380952" style="1" customWidth="1"/>
-    <col min="16" max="16" width="15.9047619047619" style="1" customWidth="1"/>
-    <col min="17" max="17" width="21.1809523809524" style="1" customWidth="1"/>
-    <col min="18" max="18" width="16.2857142857143" style="1" customWidth="1"/>
-    <col min="19" max="21" width="19.6380952380952" style="1" customWidth="1"/>
-    <col min="22" max="16371" width="9.13333333333333" style="1"/>
-    <col min="16372" max="16384" width="9" style="2"/>
+    <col min="1" max="1" customWidth="true" style="1" width="12.1428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="11.8190476190476"/>
+    <col min="3" max="3" customWidth="true" style="1" width="17.2761904761905"/>
+    <col min="4" max="5" customWidth="true" style="1" width="34.4571428571429"/>
+    <col min="6" max="9" customWidth="true" style="1" width="34.2761904761905"/>
+    <col min="10" max="10" customWidth="true" style="1" width="15.3619047619048"/>
+    <col min="11" max="11" customWidth="true" style="1" width="34.2761904761905"/>
+    <col min="12" max="12" customWidth="true" style="1" width="14.3619047619048"/>
+    <col min="13" max="13" customWidth="true" style="1" width="16.1809523809524"/>
+    <col min="14" max="14" customWidth="true" style="1" width="19.3619047619048"/>
+    <col min="15" max="15" customWidth="true" style="1" width="19.6380952380952"/>
+    <col min="16" max="16" customWidth="true" style="1" width="15.9047619047619"/>
+    <col min="17" max="17" customWidth="true" style="1" width="21.1809523809524"/>
+    <col min="18" max="18" customWidth="true" style="1" width="16.2857142857143"/>
+    <col min="19" max="21" customWidth="true" style="1" width="19.6380952380952"/>
+    <col min="22" max="16371" style="1" width="9.13333333333333"/>
+    <col min="16372" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33 16370:16371">
@@ -5358,6 +5430,9 @@
       <c r="H11" s="1" t="s">
         <v>105</v>
       </c>
+      <c r="I11" s="1" t="s">
+        <v>106</v>
+      </c>
       <c r="J11" s="10">
         <f t="shared" ref="J11:J31" si="0">H11-I11</f>
         <v>99711</v>
@@ -5393,7 +5468,10 @@
         <v>68</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>106</v>
       </c>
       <c r="J12" s="10">
         <f t="shared" si="0"/>
@@ -5433,6 +5511,9 @@
       <c r="H13" s="1" t="s">
         <v>105</v>
       </c>
+      <c r="I13" s="1" t="s">
+        <v>106</v>
+      </c>
       <c r="J13" s="10">
         <f t="shared" si="0"/>
         <v>99711</v>
@@ -5469,7 +5550,7 @@
         <v>68</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="J14" s="10">
         <f t="shared" si="0"/>
@@ -5507,7 +5588,7 @@
         <v>68</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="J15" s="10">
         <f t="shared" si="0"/>
@@ -5545,7 +5626,7 @@
         <v>68</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="J16" s="10">
         <f t="shared" si="0"/>
@@ -5583,7 +5664,7 @@
         <v>68</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="J17" s="10">
         <f t="shared" si="0"/>
@@ -6312,7 +6393,7 @@
         <v>3</v>
       </c>
       <c r="O36" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P36" s="10">
         <f t="shared" ref="P36:P42" si="3">O36-I36</f>
@@ -6375,7 +6456,7 @@
         <v>3</v>
       </c>
       <c r="O37" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P37" s="10">
         <f t="shared" si="3"/>
@@ -6438,7 +6519,7 @@
         <v>3</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P38" s="10">
         <f t="shared" si="3"/>
@@ -6501,7 +6582,7 @@
         <v>3</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P39" s="10">
         <f t="shared" si="3"/>
@@ -6564,7 +6645,7 @@
         <v>3</v>
       </c>
       <c r="O40" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P40" s="10">
         <f t="shared" si="3"/>
@@ -6627,7 +6708,7 @@
         <v>3</v>
       </c>
       <c r="O41" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P41" s="10">
         <f t="shared" si="3"/>
@@ -6690,7 +6771,7 @@
         <v>3</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P42" s="10">
         <f t="shared" si="3"/>
@@ -6866,7 +6947,7 @@
         <v>3</v>
       </c>
       <c r="O46" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P46" s="10">
         <f t="shared" ref="P46:P52" si="7">O46-I46</f>
@@ -6929,7 +7010,7 @@
         <v>3</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P47" s="10">
         <f t="shared" si="7"/>
@@ -6992,7 +7073,7 @@
         <v>3</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P48" s="10">
         <f t="shared" si="7"/>
@@ -7055,7 +7136,7 @@
         <v>3</v>
       </c>
       <c r="O49" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P49" s="10">
         <f t="shared" si="7"/>
@@ -7118,7 +7199,7 @@
         <v>3</v>
       </c>
       <c r="O50" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P50" s="10">
         <f t="shared" si="7"/>
@@ -7181,7 +7262,7 @@
         <v>3</v>
       </c>
       <c r="O51" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P51" s="10">
         <f t="shared" si="7"/>
@@ -7244,7 +7325,7 @@
         <v>3</v>
       </c>
       <c r="O52" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P52" s="10">
         <f t="shared" si="7"/>
@@ -7470,7 +7551,7 @@
         <v>3</v>
       </c>
       <c r="O57" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P57" s="10">
         <f t="shared" ref="P57:P63" si="11">O57-I57</f>
@@ -7533,7 +7614,7 @@
         <v>3</v>
       </c>
       <c r="O58" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P58" s="10">
         <f t="shared" si="11"/>
@@ -7596,7 +7677,7 @@
         <v>3</v>
       </c>
       <c r="O59" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P59" s="10">
         <f t="shared" si="11"/>
@@ -7659,7 +7740,7 @@
         <v>3</v>
       </c>
       <c r="O60" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P60" s="10">
         <f t="shared" si="11"/>
@@ -7722,7 +7803,7 @@
         <v>3</v>
       </c>
       <c r="O61" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P61" s="10">
         <f t="shared" si="11"/>
@@ -7785,7 +7866,7 @@
         <v>3</v>
       </c>
       <c r="O62" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P62" s="10">
         <f t="shared" si="11"/>
@@ -7848,7 +7929,7 @@
         <v>3</v>
       </c>
       <c r="O63" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="P63" s="10">
         <f t="shared" si="11"/>
@@ -8006,27 +8087,27 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:XEQ44"/>
+  <dimension ref="A1:XEQ42"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="12.1428571428571" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.8190476190476" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.2761904761905" style="1" customWidth="1"/>
-    <col min="4" max="5" width="34.4571428571429" style="1" customWidth="1"/>
-    <col min="6" max="6" width="42.2857142857143" style="1" customWidth="1"/>
-    <col min="7" max="9" width="34.2761904761905" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15.3619047619048" style="1" customWidth="1"/>
-    <col min="11" max="11" width="34.2761904761905" style="1" customWidth="1"/>
-    <col min="12" max="12" width="14.3619047619048" style="1" customWidth="1"/>
-    <col min="13" max="13" width="16.1809523809524" style="1" customWidth="1"/>
-    <col min="14" max="14" width="19.3619047619048" style="1" customWidth="1"/>
-    <col min="15" max="15" width="19.6380952380952" style="1" customWidth="1"/>
-    <col min="16" max="16" width="15.9047619047619" style="1" customWidth="1"/>
-    <col min="17" max="17" width="21.1809523809524" style="1" customWidth="1"/>
-    <col min="18" max="18" width="16.2857142857143" style="1" customWidth="1"/>
-    <col min="19" max="21" width="19.6380952380952" style="1" customWidth="1"/>
-    <col min="22" max="16371" width="9.13333333333333" style="1"/>
-    <col min="16372" max="16384" width="9" style="2"/>
+    <col min="1" max="1" customWidth="true" style="1" width="12.1428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="11.8190476190476"/>
+    <col min="3" max="3" customWidth="true" style="1" width="17.2761904761905"/>
+    <col min="4" max="5" customWidth="true" style="1" width="34.4571428571429"/>
+    <col min="6" max="6" customWidth="true" style="1" width="42.2857142857143"/>
+    <col min="7" max="9" customWidth="true" style="1" width="34.2761904761905"/>
+    <col min="10" max="10" customWidth="true" style="1" width="15.3619047619048"/>
+    <col min="11" max="11" customWidth="true" style="1" width="34.2761904761905"/>
+    <col min="12" max="12" customWidth="true" style="1" width="14.3619047619048"/>
+    <col min="13" max="13" customWidth="true" style="1" width="16.1809523809524"/>
+    <col min="14" max="14" customWidth="true" style="1" width="19.3619047619048"/>
+    <col min="15" max="15" customWidth="true" style="1" width="19.6380952380952"/>
+    <col min="16" max="16" customWidth="true" style="1" width="15.9047619047619"/>
+    <col min="17" max="17" customWidth="true" style="1" width="21.1809523809524"/>
+    <col min="18" max="18" customWidth="true" style="1" width="16.2857142857143"/>
+    <col min="19" max="21" customWidth="true" style="1" width="19.6380952380952"/>
+    <col min="22" max="16371" style="1" width="9.13333333333333"/>
+    <col min="16372" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33 16370:16371">
@@ -8103,10 +8184,10 @@
         <v>16</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="G3" s="25" t="s">
         <v>19</v>
@@ -8114,22 +8195,22 @@
       <c r="H3" s="8">
         <v>3</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>104</v>
+      <c r="I3" t="s" s="1">
+        <v>111</v>
       </c>
       <c r="J3" s="10">
         <f>I3+H3</f>
         <v>9</v>
       </c>
-      <c r="K3" s="1">
-        <v>2100</v>
+      <c r="K3" t="s" s="1">
+        <v>112</v>
       </c>
       <c r="L3" s="10">
-        <f>(K3+L29)/2</f>
+        <f>(K3+L27)/2</f>
         <v>1050</v>
       </c>
       <c r="M3" s="11">
-        <f>L29</f>
+        <f>L27</f>
         <v>0</v>
       </c>
       <c r="XEP3" s="2"/>
@@ -8293,147 +8374,146 @@
       <c r="AG6" s="10"/>
     </row>
     <row r="7" spans="1:33 16370:16371">
-      <c r="A7" s="10">
+      <c r="A7" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+    </row>
+    <row r="8" spans="1:33 16370:16371">
+      <c r="A8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="1:33 16370:16371">
+      <c r="A9" s="10">
+        <v>1</v>
+      </c>
+      <c r="B9" s="10">
+        <v>1</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="I9" t="s" s="1">
+        <v>104</v>
+      </c>
+      <c r="J9" s="10">
+        <f t="shared" ref="J9:J14" si="0">H9-I9</f>
+        <v>99711</v>
+      </c>
+      <c r="K9" s="10">
+        <v>1</v>
+      </c>
+      <c r="L9" s="10">
+        <f>H3</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:33 16370:16371">
+      <c r="A10" s="10">
+        <v>1</v>
+      </c>
+      <c r="B10" s="10">
         <v>2</v>
       </c>
-      <c r="B7" s="10">
-        <v>2</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="I7" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="J7" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="K7" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="L7" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="M7" s="13"/>
-      <c r="AG7" s="1">
-        <f>AG6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:33 16370:16371">
-      <c r="A8" s="10">
-        <v>3</v>
-      </c>
-      <c r="B8" s="10">
-        <v>3</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="H8" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="I8" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="J8" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="K8" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="L8" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="M8" s="13"/>
-    </row>
-    <row r="9" spans="1:33 16370:16371">
-      <c r="A9" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
-    </row>
-    <row r="10" spans="1:33 16370:16371">
-      <c r="A10" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="L10" s="7" t="s">
-        <v>66</v>
-      </c>
+      <c r="C10" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="I10" t="s" s="1">
+        <v>104</v>
+      </c>
+      <c r="J10" s="10">
+        <f t="shared" si="0"/>
+        <v>99711</v>
+      </c>
+      <c r="K10" s="10">
+        <v>1</v>
+      </c>
+      <c r="L10" s="10">
+        <f>H3</f>
+        <v>3</v>
+      </c>
+      <c r="M10" s="13"/>
     </row>
     <row r="11" spans="1:33 16370:16371">
       <c r="A11" s="10">
         <v>1</v>
       </c>
       <c r="B11" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>46</v>
@@ -8441,8 +8521,8 @@
       <c r="D11" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="24" t="s">
-        <v>70</v>
+      <c r="E11" s="15" t="s">
+        <v>71</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>14</v>
@@ -8450,11 +8530,14 @@
       <c r="G11" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>105</v>
+      <c r="H11" t="s" s="1">
+        <v>153</v>
+      </c>
+      <c r="I11" t="s" s="1">
+        <v>104</v>
       </c>
       <c r="J11" s="10">
-        <f>H11-I11</f>
+        <f t="shared" si="0"/>
         <v>99711</v>
       </c>
       <c r="K11" s="10">
@@ -8464,13 +8547,14 @@
         <f>H3</f>
         <v>3</v>
       </c>
+      <c r="M11" s="13"/>
     </row>
     <row r="12" spans="1:33 16370:16371">
       <c r="A12" s="10">
         <v>1</v>
       </c>
       <c r="B12" s="10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>46</v>
@@ -8479,7 +8563,7 @@
         <v>47</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="F12" s="10" t="s">
         <v>14</v>
@@ -8487,11 +8571,14 @@
       <c r="G12" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>105</v>
+      <c r="H12" t="s" s="1">
+        <v>153</v>
+      </c>
+      <c r="I12" t="s" s="1">
+        <v>104</v>
       </c>
       <c r="J12" s="10">
-        <f>H12-I12</f>
+        <f t="shared" si="0"/>
         <v>99711</v>
       </c>
       <c r="K12" s="10">
@@ -8508,7 +8595,7 @@
         <v>1</v>
       </c>
       <c r="B13" s="10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>46</v>
@@ -8517,7 +8604,7 @@
         <v>47</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F13" s="10" t="s">
         <v>14</v>
@@ -8525,11 +8612,14 @@
       <c r="G13" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="H13" s="1" t="s">
-        <v>105</v>
+      <c r="H13" t="s" s="1">
+        <v>153</v>
+      </c>
+      <c r="I13" t="s" s="1">
+        <v>104</v>
       </c>
       <c r="J13" s="10">
-        <f>H13-I13</f>
+        <f t="shared" si="0"/>
         <v>99711</v>
       </c>
       <c r="K13" s="10">
@@ -8546,7 +8636,7 @@
         <v>1</v>
       </c>
       <c r="B14" s="10">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>46</v>
@@ -8555,7 +8645,7 @@
         <v>47</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F14" s="10" t="s">
         <v>14</v>
@@ -8563,11 +8653,14 @@
       <c r="G14" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>105</v>
+      <c r="H14" t="s" s="1">
+        <v>153</v>
+      </c>
+      <c r="I14" t="s" s="1">
+        <v>104</v>
       </c>
       <c r="J14" s="10">
-        <f>H14-I14</f>
+        <f t="shared" si="0"/>
         <v>99711</v>
       </c>
       <c r="K14" s="10">
@@ -8580,207 +8673,257 @@
       <c r="M14" s="13"/>
     </row>
     <row r="15" spans="1:33 16370:16371">
-      <c r="A15" s="10">
-        <v>1</v>
-      </c>
-      <c r="B15" s="10">
-        <v>5</v>
-      </c>
-      <c r="C15" s="10" t="s">
+      <c r="A15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="13"/>
+      <c r="N15" s="13"/>
+      <c r="O15" s="13"/>
+      <c r="P15" s="13"/>
+      <c r="Q15" s="13"/>
+      <c r="R15" s="13"/>
+    </row>
+    <row r="16" spans="1:33 16370:16371">
+      <c r="A16" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="12"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
+      <c r="O16" s="12"/>
+      <c r="P16" s="12"/>
+      <c r="Q16" s="12"/>
+      <c r="R16" s="12"/>
+    </row>
+    <row r="17" spans="1:19">
+      <c r="A17" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18"/>
+      <c r="L17" s="18"/>
+      <c r="M17" s="18"/>
+      <c r="N17" s="18"/>
+      <c r="O17" s="18"/>
+      <c r="P17" s="18"/>
+      <c r="Q17" s="18"/>
+      <c r="R17" s="19"/>
+    </row>
+    <row r="18" spans="1:19">
+      <c r="A18" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="O18" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="P18" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q18" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="R18" s="7" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19">
+      <c r="A19" s="10">
+        <v>1</v>
+      </c>
+      <c r="B19" s="10">
+        <v>1</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D19" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="E15" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="J15" s="10">
-        <f>H15-I15</f>
-        <v>99711</v>
-      </c>
-      <c r="K15" s="10">
-        <v>1</v>
-      </c>
-      <c r="L15" s="10">
-        <f>H3</f>
-        <v>3</v>
-      </c>
-      <c r="M15" s="13"/>
-    </row>
-    <row r="16" spans="1:33 16370:16371">
-      <c r="A16" s="10">
-        <v>1</v>
-      </c>
-      <c r="B16" s="10">
-        <v>6</v>
-      </c>
-      <c r="C16" s="10" t="s">
+      <c r="E19" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H19" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="I19" s="10">
+        <f>H3</f>
+        <v>3</v>
+      </c>
+      <c r="J19" s="10">
+        <f>H3</f>
+        <v>3</v>
+      </c>
+      <c r="K19" s="10">
+        <f>H3</f>
+        <v>3</v>
+      </c>
+      <c r="L19" s="10">
+        <v>100</v>
+      </c>
+      <c r="M19" s="10">
+        <f t="shared" ref="M19:M25" si="1">L19*K19</f>
+        <v>300</v>
+      </c>
+      <c r="N19" s="10">
+        <v>3</v>
+      </c>
+      <c r="O19" t="s" s="1">
+        <v>153</v>
+      </c>
+      <c r="P19" s="10">
+        <f t="shared" ref="P19:P25" si="2">O19-I19</f>
+        <v>99708</v>
+      </c>
+      <c r="Q19" s="10">
+        <f t="shared" ref="Q19:Q25" si="3">-I19</f>
+        <v>-3</v>
+      </c>
+      <c r="R19" s="10">
+        <f t="shared" ref="R19:R25" si="4">I19</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19">
+      <c r="A20" s="10">
+        <v>1</v>
+      </c>
+      <c r="B20" s="10">
+        <v>2</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D20" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="E16" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="J16" s="10">
-        <f>H16-I16</f>
-        <v>99711</v>
-      </c>
-      <c r="K16" s="10">
-        <v>1</v>
-      </c>
-      <c r="L16" s="10">
-        <f>H3</f>
-        <v>3</v>
-      </c>
-      <c r="M16" s="13"/>
-    </row>
-    <row r="17" spans="1:18">
-      <c r="A17" s="16"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="16"/>
-      <c r="K17" s="16"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="13"/>
-      <c r="O17" s="13"/>
-      <c r="P17" s="13"/>
-      <c r="Q17" s="13"/>
-      <c r="R17" s="13"/>
-    </row>
-    <row r="18" spans="1:18">
-      <c r="A18" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="12"/>
-      <c r="M18" s="12"/>
-      <c r="N18" s="12"/>
-      <c r="O18" s="12"/>
-      <c r="P18" s="12"/>
-      <c r="Q18" s="12"/>
-      <c r="R18" s="12"/>
-    </row>
-    <row r="19" spans="1:18">
-      <c r="A19" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18"/>
-      <c r="M19" s="18"/>
-      <c r="N19" s="18"/>
-      <c r="O19" s="18"/>
-      <c r="P19" s="18"/>
-      <c r="Q19" s="18"/>
-      <c r="R19" s="19"/>
-    </row>
-    <row r="20" spans="1:18">
-      <c r="A20" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="I20" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="J20" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="K20" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="L20" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="M20" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="N20" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="O20" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="P20" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q20" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="R20" s="7" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="21" spans="1:18">
+      <c r="E20" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H20" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="I20" s="10">
+        <f>H3</f>
+        <v>3</v>
+      </c>
+      <c r="J20" s="10">
+        <f>H3</f>
+        <v>3</v>
+      </c>
+      <c r="K20" s="10">
+        <f>H3</f>
+        <v>3</v>
+      </c>
+      <c r="L20" s="10">
+        <v>100</v>
+      </c>
+      <c r="M20" s="10">
+        <f t="shared" si="1"/>
+        <v>300</v>
+      </c>
+      <c r="N20" s="10">
+        <v>3</v>
+      </c>
+      <c r="O20" t="s" s="1">
+        <v>154</v>
+      </c>
+      <c r="P20" s="10">
+        <f t="shared" si="2"/>
+        <v>99708</v>
+      </c>
+      <c r="Q20" s="10">
+        <f t="shared" si="3"/>
+        <v>-3</v>
+      </c>
+      <c r="R20" s="10">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19">
       <c r="A21" s="10">
         <v>1</v>
       </c>
       <c r="B21" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C21" s="10" t="s">
         <v>46</v>
@@ -8789,7 +8932,7 @@
         <v>47</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>14</v>
@@ -8816,34 +8959,34 @@
         <v>100</v>
       </c>
       <c r="M21" s="10">
-        <f t="shared" ref="M21:M27" si="0">L21*K21</f>
+        <f t="shared" si="1"/>
         <v>300</v>
       </c>
       <c r="N21" s="10">
         <v>3</v>
       </c>
-      <c r="O21" s="1" t="s">
-        <v>105</v>
+      <c r="O21" t="s" s="1">
+        <v>153</v>
       </c>
       <c r="P21" s="10">
-        <f t="shared" ref="P21:P27" si="1">O21-I21</f>
+        <f t="shared" si="2"/>
         <v>99708</v>
       </c>
       <c r="Q21" s="10">
-        <f t="shared" ref="Q21:Q27" si="2">-I21</f>
+        <f t="shared" si="3"/>
         <v>-3</v>
       </c>
       <c r="R21" s="10">
-        <f t="shared" ref="R21:R27" si="3">I21</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:18">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19">
       <c r="A22" s="10">
         <v>1</v>
       </c>
       <c r="B22" s="10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C22" s="10" t="s">
         <v>46</v>
@@ -8852,7 +8995,7 @@
         <v>47</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="F22" s="10" t="s">
         <v>14</v>
@@ -8879,34 +9022,34 @@
         <v>100</v>
       </c>
       <c r="M22" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>300</v>
       </c>
       <c r="N22" s="10">
         <v>3</v>
       </c>
-      <c r="O22" s="1" t="s">
-        <v>105</v>
+      <c r="O22" t="s" s="1">
+        <v>153</v>
       </c>
       <c r="P22" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>99708</v>
       </c>
       <c r="Q22" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-3</v>
       </c>
       <c r="R22" s="10">
-        <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:18">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19">
       <c r="A23" s="10">
         <v>1</v>
       </c>
       <c r="B23" s="10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C23" s="10" t="s">
         <v>46</v>
@@ -8915,7 +9058,7 @@
         <v>47</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F23" s="10" t="s">
         <v>14</v>
@@ -8942,34 +9085,34 @@
         <v>100</v>
       </c>
       <c r="M23" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>300</v>
       </c>
       <c r="N23" s="10">
         <v>3</v>
       </c>
-      <c r="O23" s="1" t="s">
-        <v>105</v>
+      <c r="O23" t="s" s="1">
+        <v>153</v>
       </c>
       <c r="P23" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>99708</v>
       </c>
       <c r="Q23" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-3</v>
       </c>
       <c r="R23" s="10">
-        <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:18">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19">
       <c r="A24" s="10">
         <v>1</v>
       </c>
       <c r="B24" s="10">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C24" s="10" t="s">
         <v>46</v>
@@ -8978,7 +9121,7 @@
         <v>47</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F24" s="10" t="s">
         <v>14</v>
@@ -9005,299 +9148,301 @@
         <v>100</v>
       </c>
       <c r="M24" s="10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>300</v>
       </c>
       <c r="N24" s="10">
         <v>3</v>
       </c>
-      <c r="O24" s="1" t="s">
-        <v>105</v>
+      <c r="O24" t="s" s="1">
+        <v>153</v>
       </c>
       <c r="P24" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>99708</v>
       </c>
       <c r="Q24" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-3</v>
       </c>
       <c r="R24" s="10">
-        <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:18">
-      <c r="A25" s="10">
-        <v>1</v>
-      </c>
-      <c r="B25" s="10">
-        <v>5</v>
-      </c>
-      <c r="C25" s="10" t="s">
+        <f t="shared" si="4"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19">
+      <c r="A25" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="B25" s="20">
+        <v>1</v>
+      </c>
+      <c r="C25" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="20"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="I25" s="20">
+        <v>3</v>
+      </c>
+      <c r="J25" s="20">
+        <v>3</v>
+      </c>
+      <c r="K25" s="20"/>
+      <c r="L25" s="22">
+        <f>SUM(L19:L24)</f>
+        <v>600</v>
+      </c>
+      <c r="M25" s="22">
+        <f>SUM(M19:M24)</f>
+        <v>1800</v>
+      </c>
+      <c r="N25" s="22">
+        <v>100</v>
+      </c>
+      <c r="O25" s="1"/>
+      <c r="P25" s="20"/>
+      <c r="Q25" s="20"/>
+      <c r="R25" s="20"/>
+    </row>
+    <row r="26" spans="1:19">
+      <c r="A26" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="12"/>
+      <c r="M26" s="12"/>
+      <c r="N26" s="12"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="12"/>
+      <c r="Q26" s="12"/>
+      <c r="R26" s="12"/>
+    </row>
+    <row r="27" spans="1:19">
+      <c r="A27" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="18"/>
+      <c r="J27" s="18"/>
+      <c r="K27" s="18"/>
+      <c r="L27" s="18"/>
+      <c r="M27" s="18"/>
+      <c r="N27" s="18"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="18"/>
+      <c r="Q27" s="18"/>
+      <c r="R27" s="19"/>
+    </row>
+    <row r="28" spans="1:19">
+      <c r="A28" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="J28" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="K28" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="L28" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="M28" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="N28" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="O28" s="1"/>
+      <c r="P28" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q28" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="R28" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="S28" s="7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19">
+      <c r="A29" s="10">
+        <v>1</v>
+      </c>
+      <c r="B29" s="10">
+        <v>1</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="E25" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="F25" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="G25" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="H25" s="14" t="s">
+      <c r="E29" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F29" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H29" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="I25" s="10">
-        <f>H3</f>
-        <v>3</v>
-      </c>
-      <c r="J25" s="10">
-        <f>H3</f>
-        <v>3</v>
-      </c>
-      <c r="K25" s="10">
-        <f>H3</f>
-        <v>3</v>
-      </c>
-      <c r="L25" s="10">
+      <c r="I29" s="10">
+        <v>3</v>
+      </c>
+      <c r="J29" s="10">
+        <v>13</v>
+      </c>
+      <c r="K29" s="10">
+        <v>13</v>
+      </c>
+      <c r="L29" s="10">
         <v>100</v>
       </c>
-      <c r="M25" s="10">
-        <f t="shared" si="0"/>
-        <v>300</v>
-      </c>
-      <c r="N25" s="10">
-        <v>3</v>
-      </c>
-      <c r="O25" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="P25" s="10">
-        <f t="shared" si="1"/>
-        <v>99708</v>
-      </c>
-      <c r="Q25" s="10">
-        <f t="shared" si="2"/>
+      <c r="M29" s="10">
+        <f t="shared" ref="M29:M35" si="5">L29*K29</f>
+        <v>1300</v>
+      </c>
+      <c r="N29" s="10">
+        <v>3</v>
+      </c>
+      <c r="O29" t="s" s="1">
+        <v>153</v>
+      </c>
+      <c r="P29" s="10">
+        <f>O29-S29</f>
+        <v>99627</v>
+      </c>
+      <c r="Q29" s="10">
+        <f t="shared" ref="Q29:Q35" si="6">-I29</f>
         <v>-3</v>
       </c>
-      <c r="R25" s="10">
-        <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:18">
-      <c r="A26" s="10">
-        <v>1</v>
-      </c>
-      <c r="B26" s="10">
-        <v>6</v>
-      </c>
-      <c r="C26" s="10" t="s">
+      <c r="R29" s="10">
+        <f t="shared" ref="R29:R35" si="7">I29</f>
+        <v>3</v>
+      </c>
+      <c r="S29" s="10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19">
+      <c r="A30" s="10">
+        <v>1</v>
+      </c>
+      <c r="B30" s="10">
+        <v>2</v>
+      </c>
+      <c r="C30" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D30" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="E26" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="F26" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="H26" s="14" t="s">
+      <c r="E30" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G30" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H30" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="I26" s="10">
-        <f>H3</f>
-        <v>3</v>
-      </c>
-      <c r="J26" s="10">
-        <f>H3</f>
-        <v>3</v>
-      </c>
-      <c r="K26" s="10">
-        <f>H3</f>
-        <v>3</v>
-      </c>
-      <c r="L26" s="10">
+      <c r="I30" s="10">
+        <v>3</v>
+      </c>
+      <c r="J30" s="10">
+        <v>13</v>
+      </c>
+      <c r="K30" s="10">
+        <v>13</v>
+      </c>
+      <c r="L30" s="10">
         <v>100</v>
       </c>
-      <c r="M26" s="10">
-        <f t="shared" si="0"/>
-        <v>300</v>
-      </c>
-      <c r="N26" s="10">
-        <v>3</v>
-      </c>
-      <c r="O26" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="P26" s="10">
-        <f t="shared" si="1"/>
-        <v>99708</v>
-      </c>
-      <c r="Q26" s="10">
-        <f t="shared" si="2"/>
+      <c r="M30" s="10">
+        <f t="shared" si="5"/>
+        <v>1300</v>
+      </c>
+      <c r="N30" s="10">
+        <v>3</v>
+      </c>
+      <c r="O30" t="s" s="1">
+        <v>154</v>
+      </c>
+      <c r="P30" s="10">
+        <f t="shared" ref="P30:P35" si="8">O30-S30</f>
+        <v>99637</v>
+      </c>
+      <c r="Q30" s="10">
+        <f t="shared" si="6"/>
         <v>-3</v>
       </c>
-      <c r="R26" s="10">
-        <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:18">
-      <c r="A27" s="20" t="s">
-        <v>95</v>
-      </c>
-      <c r="B27" s="20">
-        <v>1</v>
-      </c>
-      <c r="C27" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="D27" s="20"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="I27" s="20">
-        <v>3</v>
-      </c>
-      <c r="J27" s="20">
-        <v>3</v>
-      </c>
-      <c r="K27" s="20"/>
-      <c r="L27" s="22">
-        <f>SUM(L21:L26)</f>
-        <v>600</v>
-      </c>
-      <c r="M27" s="22">
-        <f>SUM(M21:M26)</f>
-        <v>1800</v>
-      </c>
-      <c r="N27" s="22">
-        <v>100</v>
-      </c>
-      <c r="P27" s="20"/>
-      <c r="Q27" s="20"/>
-      <c r="R27" s="20"/>
-    </row>
-    <row r="28" spans="1:18">
-      <c r="A28" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="12"/>
-      <c r="I28" s="12"/>
-      <c r="J28" s="12"/>
-      <c r="K28" s="12"/>
-      <c r="L28" s="12"/>
-      <c r="M28" s="12"/>
-      <c r="N28" s="12"/>
-      <c r="O28" s="12"/>
-      <c r="P28" s="12"/>
-      <c r="Q28" s="12"/>
-      <c r="R28" s="12"/>
-    </row>
-    <row r="29" spans="1:18">
-      <c r="A29" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
-      <c r="G29" s="18"/>
-      <c r="H29" s="18"/>
-      <c r="I29" s="18"/>
-      <c r="J29" s="18"/>
-      <c r="K29" s="18"/>
-      <c r="L29" s="18"/>
-      <c r="M29" s="18"/>
-      <c r="N29" s="18"/>
-      <c r="O29" s="18"/>
-      <c r="P29" s="18"/>
-      <c r="Q29" s="18"/>
-      <c r="R29" s="19"/>
-    </row>
-    <row r="30" spans="1:18">
-      <c r="A30" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E30" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="I30" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="J30" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="K30" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="L30" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="M30" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="N30" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="O30" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="P30" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q30" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="R30" s="7" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="31" spans="1:18">
+      <c r="R30" s="10">
+        <f t="shared" si="7"/>
+        <v>3</v>
+      </c>
+      <c r="S30" s="10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19">
       <c r="A31" s="10">
         <v>1</v>
       </c>
       <c r="B31" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C31" s="10" t="s">
         <v>46</v>
@@ -9306,7 +9451,7 @@
         <v>47</v>
       </c>
       <c r="E31" s="15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>14</v>
@@ -9317,50 +9462,50 @@
       <c r="H31" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="I31" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="J31" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="K31" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
+      <c r="I31" s="10">
+        <v>3</v>
+      </c>
+      <c r="J31" s="10">
+        <v>13</v>
+      </c>
+      <c r="K31" s="10">
+        <v>13</v>
       </c>
       <c r="L31" s="10">
         <v>100</v>
       </c>
       <c r="M31" s="10">
-        <f t="shared" ref="M31:M37" si="4">L31*K31</f>
-        <v>9971100</v>
+        <f t="shared" si="5"/>
+        <v>1300</v>
       </c>
       <c r="N31" s="10">
-        <v>13</v>
-      </c>
-      <c r="O31" s="1" t="s">
-        <v>105</v>
+        <v>3</v>
+      </c>
+      <c r="O31" t="s" s="1">
+        <v>153</v>
       </c>
       <c r="P31" s="10">
-        <f t="shared" ref="P31:P37" si="5">O31-I31</f>
-        <v>0</v>
+        <f t="shared" si="8"/>
+        <v>99627</v>
       </c>
       <c r="Q31" s="10">
-        <f t="shared" ref="Q31:Q37" si="6">-I31</f>
-        <v>-99711</v>
-      </c>
-      <c r="R31" s="10" t="str">
-        <f t="shared" ref="R31:R37" si="7">I31</f>
-        <v>99711</v>
-      </c>
-    </row>
-    <row r="32" spans="1:18">
+        <f t="shared" si="6"/>
+        <v>-3</v>
+      </c>
+      <c r="R31" s="10">
+        <f t="shared" si="7"/>
+        <v>3</v>
+      </c>
+      <c r="S31" s="10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19">
       <c r="A32" s="10">
         <v>1</v>
       </c>
       <c r="B32" s="10">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C32" s="10" t="s">
         <v>46</v>
@@ -9369,7 +9514,7 @@
         <v>47</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="F32" s="10" t="s">
         <v>14</v>
@@ -9380,50 +9525,50 @@
       <c r="H32" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="I32" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="J32" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="K32" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
+      <c r="I32" s="10">
+        <v>3</v>
+      </c>
+      <c r="J32" s="10">
+        <v>13</v>
+      </c>
+      <c r="K32" s="10">
+        <v>13</v>
       </c>
       <c r="L32" s="10">
         <v>100</v>
       </c>
       <c r="M32" s="10">
-        <f t="shared" si="4"/>
-        <v>9971100</v>
+        <f t="shared" si="5"/>
+        <v>1300</v>
       </c>
       <c r="N32" s="10">
-        <v>13</v>
-      </c>
-      <c r="O32" s="1" t="s">
-        <v>105</v>
+        <v>3</v>
+      </c>
+      <c r="O32" t="s" s="1">
+        <v>153</v>
       </c>
       <c r="P32" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f t="shared" si="8"/>
+        <v>99627</v>
       </c>
       <c r="Q32" s="10">
         <f t="shared" si="6"/>
-        <v>-99711</v>
-      </c>
-      <c r="R32" s="10" t="str">
+        <v>-3</v>
+      </c>
+      <c r="R32" s="10">
         <f t="shared" si="7"/>
-        <v>99711</v>
-      </c>
-    </row>
-    <row r="33" spans="1:18">
+        <v>3</v>
+      </c>
+      <c r="S32" s="10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19">
       <c r="A33" s="10">
         <v>1</v>
       </c>
       <c r="B33" s="10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C33" s="10" t="s">
         <v>46</v>
@@ -9432,7 +9577,7 @@
         <v>47</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>14</v>
@@ -9443,50 +9588,50 @@
       <c r="H33" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="I33" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="J33" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="K33" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
+      <c r="I33" s="10">
+        <v>3</v>
+      </c>
+      <c r="J33" s="10">
+        <v>13</v>
+      </c>
+      <c r="K33" s="10">
+        <v>13</v>
       </c>
       <c r="L33" s="10">
         <v>100</v>
       </c>
       <c r="M33" s="10">
-        <f t="shared" si="4"/>
-        <v>9971100</v>
+        <f t="shared" si="5"/>
+        <v>1300</v>
       </c>
       <c r="N33" s="10">
-        <v>13</v>
-      </c>
-      <c r="O33" s="1" t="s">
-        <v>105</v>
+        <v>3</v>
+      </c>
+      <c r="O33" t="s" s="1">
+        <v>153</v>
       </c>
       <c r="P33" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f t="shared" si="8"/>
+        <v>99627</v>
       </c>
       <c r="Q33" s="10">
         <f t="shared" si="6"/>
-        <v>-99711</v>
-      </c>
-      <c r="R33" s="10" t="str">
+        <v>-3</v>
+      </c>
+      <c r="R33" s="10">
         <f t="shared" si="7"/>
-        <v>99711</v>
-      </c>
-    </row>
-    <row r="34" spans="1:18">
+        <v>3</v>
+      </c>
+      <c r="S33" s="10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19">
       <c r="A34" s="10">
         <v>1</v>
       </c>
       <c r="B34" s="10">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C34" s="10" t="s">
         <v>46</v>
@@ -9495,7 +9640,7 @@
         <v>47</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F34" s="10" t="s">
         <v>14</v>
@@ -9506,50 +9651,50 @@
       <c r="H34" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="I34" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="J34" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="K34" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
+      <c r="I34" s="10">
+        <v>3</v>
+      </c>
+      <c r="J34" s="10">
+        <v>13</v>
+      </c>
+      <c r="K34" s="10">
+        <v>13</v>
       </c>
       <c r="L34" s="10">
         <v>100</v>
       </c>
       <c r="M34" s="10">
-        <f t="shared" si="4"/>
-        <v>9971100</v>
+        <f t="shared" si="5"/>
+        <v>1300</v>
       </c>
       <c r="N34" s="10">
-        <v>13</v>
-      </c>
-      <c r="O34" s="1" t="s">
-        <v>105</v>
+        <v>3</v>
+      </c>
+      <c r="O34" t="s" s="1">
+        <v>153</v>
       </c>
       <c r="P34" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f t="shared" si="8"/>
+        <v>99627</v>
       </c>
       <c r="Q34" s="10">
         <f t="shared" si="6"/>
-        <v>-99711</v>
-      </c>
-      <c r="R34" s="10" t="str">
+        <v>-3</v>
+      </c>
+      <c r="R34" s="10">
         <f t="shared" si="7"/>
-        <v>99711</v>
-      </c>
-    </row>
-    <row r="35" spans="1:18">
+        <v>3</v>
+      </c>
+      <c r="S34" s="10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19">
       <c r="A35" s="10">
         <v>1</v>
       </c>
       <c r="B35" s="10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C35" s="10" t="s">
         <v>46</v>
@@ -9558,7 +9703,7 @@
         <v>47</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>14</v>
@@ -9569,50 +9714,50 @@
       <c r="H35" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="I35" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="J35" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="K35" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
+      <c r="I35" s="10">
+        <v>0</v>
+      </c>
+      <c r="J35" s="10">
+        <v>13</v>
+      </c>
+      <c r="K35" s="10">
+        <v>13</v>
       </c>
       <c r="L35" s="10">
         <v>100</v>
       </c>
       <c r="M35" s="10">
-        <f t="shared" si="4"/>
-        <v>9971100</v>
+        <f t="shared" si="5"/>
+        <v>1300</v>
       </c>
       <c r="N35" s="10">
-        <v>13</v>
-      </c>
-      <c r="O35" s="1" t="s">
-        <v>105</v>
+        <v>0</v>
+      </c>
+      <c r="O35" t="s" s="1">
+        <v>138</v>
       </c>
       <c r="P35" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f t="shared" si="8"/>
+        <v>99695</v>
       </c>
       <c r="Q35" s="10">
         <f t="shared" si="6"/>
-        <v>-99711</v>
-      </c>
-      <c r="R35" s="10" t="str">
+        <v>0</v>
+      </c>
+      <c r="R35" s="10">
         <f t="shared" si="7"/>
-        <v>99711</v>
-      </c>
-    </row>
-    <row r="36" spans="1:18">
+        <v>0</v>
+      </c>
+      <c r="S35" s="10">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19">
       <c r="A36" s="10">
         <v>1</v>
       </c>
       <c r="B36" s="10">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C36" s="10" t="s">
         <v>46</v>
@@ -9620,217 +9765,106 @@
       <c r="D36" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="E36" s="15" t="s">
-        <v>74</v>
-      </c>
+      <c r="E36" s="15"/>
       <c r="F36" s="10" t="s">
         <v>14</v>
       </c>
       <c r="G36" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="H36" s="14" t="s">
+      <c r="H36" s="14"/>
+      <c r="I36" s="10"/>
+      <c r="J36" s="10"/>
+      <c r="K36" s="10"/>
+      <c r="L36" s="10"/>
+      <c r="M36" s="10"/>
+      <c r="N36" s="10"/>
+      <c r="O36" s="1"/>
+      <c r="P36" s="10"/>
+      <c r="Q36" s="10"/>
+      <c r="R36" s="10"/>
+      <c r="S36" s="10"/>
+    </row>
+    <row r="37" spans="1:19">
+      <c r="A37" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="B37" s="20">
+        <v>1</v>
+      </c>
+      <c r="C37" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D37" s="20"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="20"/>
+      <c r="G37" s="20"/>
+      <c r="H37" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="I36" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="J36" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="K36" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="L36" s="10">
+      <c r="I37" s="20">
+        <v>3</v>
+      </c>
+      <c r="J37" s="20">
+        <v>3</v>
+      </c>
+      <c r="K37" s="20"/>
+      <c r="L37" s="22">
+        <f>SUM(L29:L35)</f>
+        <v>700</v>
+      </c>
+      <c r="M37" s="22">
+        <f>SUM(M29:M35)</f>
+        <v>9100</v>
+      </c>
+      <c r="N37" s="22">
         <v>100</v>
       </c>
-      <c r="M36" s="10">
-        <f t="shared" si="4"/>
-        <v>9971100</v>
-      </c>
-      <c r="N36" s="10">
-        <v>13</v>
-      </c>
-      <c r="O36" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="P36" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q36" s="10">
-        <f t="shared" si="6"/>
-        <v>-99711</v>
-      </c>
-      <c r="R36" s="10" t="str">
-        <f t="shared" si="7"/>
-        <v>99711</v>
-      </c>
-    </row>
-    <row r="37" spans="1:18">
-      <c r="A37" s="10">
-        <v>1</v>
-      </c>
-      <c r="B37" s="10">
-        <v>7</v>
-      </c>
-      <c r="C37" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D37" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E37" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="F37" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="G37" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="H37" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="I37" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="J37" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="K37" s="10" t="str">
-        <f>H14</f>
-        <v>99711</v>
-      </c>
-      <c r="L37" s="10">
-        <v>100</v>
-      </c>
-      <c r="M37" s="10">
-        <f t="shared" si="4"/>
-        <v>9971100</v>
-      </c>
-      <c r="N37" s="10">
-        <v>10</v>
-      </c>
-      <c r="O37" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="P37" s="10">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="Q37" s="10">
-        <f t="shared" si="6"/>
-        <v>-99711</v>
-      </c>
-      <c r="R37" s="10" t="str">
-        <f t="shared" si="7"/>
-        <v>99711</v>
-      </c>
-    </row>
-    <row r="38" spans="1:18">
-      <c r="A38" s="10">
-        <v>1</v>
-      </c>
-      <c r="B38" s="10">
-        <v>8</v>
-      </c>
-      <c r="C38" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D38" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E38" s="15"/>
-      <c r="F38" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="G38" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="H38" s="14"/>
-      <c r="I38" s="10"/>
-      <c r="J38" s="10"/>
-      <c r="K38" s="10"/>
-      <c r="L38" s="10"/>
-      <c r="M38" s="10"/>
-      <c r="N38" s="10"/>
-      <c r="P38" s="10"/>
-      <c r="Q38" s="10"/>
-      <c r="R38" s="10"/>
-    </row>
-    <row r="39" spans="1:18">
-      <c r="A39" s="20" t="s">
-        <v>95</v>
-      </c>
-      <c r="B39" s="20">
-        <v>1</v>
-      </c>
-      <c r="C39" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="D39" s="20"/>
-      <c r="E39" s="21"/>
-      <c r="F39" s="20"/>
-      <c r="G39" s="20"/>
-      <c r="H39" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="I39" s="20">
-        <v>3</v>
-      </c>
-      <c r="J39" s="20">
-        <v>3</v>
-      </c>
-      <c r="K39" s="20"/>
-      <c r="L39" s="22">
-        <f>SUM(L31:L37)</f>
-        <v>700</v>
-      </c>
-      <c r="M39" s="22">
-        <f>SUM(M31:M37)</f>
-        <v>69797700</v>
-      </c>
-      <c r="N39" s="22">
-        <v>100</v>
-      </c>
-      <c r="P39" s="20"/>
-      <c r="Q39" s="20"/>
-      <c r="R39" s="20"/>
-    </row>
-    <row r="43" spans="1:18">
-      <c r="K43" s="11" t="s">
+      <c r="O37" s="1"/>
+      <c r="P37" s="20"/>
+      <c r="Q37" s="20"/>
+      <c r="R37" s="20"/>
+      <c r="S37" s="20"/>
+    </row>
+    <row r="38">
+      <c r="O38" s="1"/>
+    </row>
+    <row r="39">
+      <c r="O39" s="1"/>
+    </row>
+    <row r="40">
+      <c r="O40" s="1"/>
+    </row>
+    <row r="41" spans="1:19">
+      <c r="K41" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="L43" s="11">
-        <f>L39/H3</f>
+      <c r="L41" s="11">
+        <f>L37/H3</f>
         <v>233.333333333333</v>
       </c>
-    </row>
-    <row r="44" spans="1:18">
-      <c r="K44" s="11" t="s">
+      <c r="O41" s="1"/>
+    </row>
+    <row r="42" spans="1:19">
+      <c r="K42" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="L44" s="11">
-        <f>L39+AG7</f>
-        <v>700</v>
-      </c>
+      <c r="L42" s="11" t="e">
+        <f>M37+#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="O42" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A4:L4"/>
     <mergeCell ref="V4:AG4"/>
-    <mergeCell ref="A9:L9"/>
-    <mergeCell ref="A18:R18"/>
-    <mergeCell ref="A19:R19"/>
-    <mergeCell ref="A28:R28"/>
-    <mergeCell ref="A29:R29"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A16:R16"/>
+    <mergeCell ref="A17:R17"/>
+    <mergeCell ref="A26:R26"/>
+    <mergeCell ref="A27:R27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -9843,23 +9877,23 @@
   <dimension ref="A1:XEQ66"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="12.1428571428571" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.8190476190476" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.2761904761905" style="1" customWidth="1"/>
-    <col min="4" max="5" width="34.4571428571429" style="1" customWidth="1"/>
-    <col min="6" max="9" width="34.2761904761905" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15.3619047619048" style="1" customWidth="1"/>
-    <col min="11" max="11" width="34.2761904761905" style="1" customWidth="1"/>
-    <col min="12" max="12" width="14.3619047619048" style="1" customWidth="1"/>
-    <col min="13" max="13" width="16.1809523809524" style="1" customWidth="1"/>
-    <col min="14" max="14" width="19.3619047619048" style="1" customWidth="1"/>
-    <col min="15" max="15" width="19.6380952380952" style="1" customWidth="1"/>
-    <col min="16" max="16" width="15.9047619047619" style="1" customWidth="1"/>
-    <col min="17" max="17" width="21.1809523809524" style="1" customWidth="1"/>
-    <col min="18" max="18" width="16.2857142857143" style="1" customWidth="1"/>
-    <col min="19" max="21" width="19.6380952380952" style="1" customWidth="1"/>
-    <col min="22" max="16371" width="9.13333333333333" style="1"/>
-    <col min="16372" max="16384" width="9" style="2"/>
+    <col min="1" max="1" customWidth="true" style="1" width="12.1428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="11.8190476190476"/>
+    <col min="3" max="3" customWidth="true" style="1" width="17.2761904761905"/>
+    <col min="4" max="5" customWidth="true" style="1" width="34.4571428571429"/>
+    <col min="6" max="9" customWidth="true" style="1" width="34.2761904761905"/>
+    <col min="10" max="10" customWidth="true" style="1" width="15.3619047619048"/>
+    <col min="11" max="11" customWidth="true" style="1" width="34.2761904761905"/>
+    <col min="12" max="12" customWidth="true" style="1" width="14.3619047619048"/>
+    <col min="13" max="13" customWidth="true" style="1" width="16.1809523809524"/>
+    <col min="14" max="14" customWidth="true" style="1" width="19.3619047619048"/>
+    <col min="15" max="15" customWidth="true" style="1" width="19.6380952380952"/>
+    <col min="16" max="16" customWidth="true" style="1" width="15.9047619047619"/>
+    <col min="17" max="17" customWidth="true" style="1" width="21.1809523809524"/>
+    <col min="18" max="18" customWidth="true" style="1" width="16.2857142857143"/>
+    <col min="19" max="21" customWidth="true" style="1" width="19.6380952380952"/>
+    <col min="22" max="16371" style="1" width="9.13333333333333"/>
+    <col min="16372" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33 16370:16371">
@@ -9936,7 +9970,7 @@
         <v>16</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>18</v>
@@ -9948,7 +9982,7 @@
         <v>3</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="J3" s="10">
         <f>I3+H3</f>
@@ -10284,10 +10318,10 @@
         <v>68</v>
       </c>
       <c r="H11" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I11" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="J11" s="10">
         <f t="shared" ref="J11:J31" si="0">H11-I11</f>
@@ -10324,10 +10358,10 @@
         <v>68</v>
       </c>
       <c r="H12" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I12" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="J12" s="10">
         <f t="shared" si="0"/>
@@ -10365,10 +10399,10 @@
         <v>68</v>
       </c>
       <c r="H13" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="J13" s="10">
         <f t="shared" si="0"/>
@@ -10406,10 +10440,10 @@
         <v>68</v>
       </c>
       <c r="H14" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="J14" s="10">
         <f t="shared" si="0"/>
@@ -10447,10 +10481,10 @@
         <v>68</v>
       </c>
       <c r="H15" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="J15" s="10">
         <f t="shared" si="0"/>
@@ -10488,10 +10522,10 @@
         <v>68</v>
       </c>
       <c r="H16" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="J16" s="10">
         <f t="shared" si="0"/>
@@ -10529,10 +10563,10 @@
         <v>68</v>
       </c>
       <c r="H17" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="I17" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="J17" s="10">
         <f t="shared" si="0"/>
@@ -10561,7 +10595,7 @@
         <v>55</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="F18" s="10" t="s">
         <v>14</v>
@@ -10574,7 +10608,7 @@
         <v>99813</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J18" s="10">
         <f t="shared" si="0"/>
@@ -10603,7 +10637,7 @@
         <v>55</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>14</v>
@@ -10616,7 +10650,7 @@
         <v>99813</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J19" s="10">
         <f t="shared" si="0"/>
@@ -10645,7 +10679,7 @@
         <v>55</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="F20" s="10" t="s">
         <v>14</v>
@@ -10658,7 +10692,7 @@
         <v>99813</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J20" s="10">
         <f t="shared" si="0"/>
@@ -10687,7 +10721,7 @@
         <v>55</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>14</v>
@@ -10700,7 +10734,7 @@
         <v>99813</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J21" s="10">
         <f t="shared" si="0"/>
@@ -10729,7 +10763,7 @@
         <v>55</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="F22" s="10" t="s">
         <v>14</v>
@@ -10742,7 +10776,7 @@
         <v>99813</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J22" s="10">
         <f t="shared" si="0"/>
@@ -10771,7 +10805,7 @@
         <v>55</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="F23" s="10" t="s">
         <v>14</v>
@@ -10784,7 +10818,7 @@
         <v>99813</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J23" s="10">
         <f t="shared" si="0"/>
@@ -10813,7 +10847,7 @@
         <v>55</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F24" s="10" t="s">
         <v>14</v>
@@ -10826,7 +10860,7 @@
         <v>99813</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J24" s="10">
         <f t="shared" si="0"/>
@@ -10855,7 +10889,7 @@
         <v>57</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>14</v>
@@ -10897,7 +10931,7 @@
         <v>57</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="F26" s="10" t="s">
         <v>14</v>
@@ -10939,7 +10973,7 @@
         <v>57</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>14</v>
@@ -10981,7 +11015,7 @@
         <v>57</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="F28" s="10" t="s">
         <v>14</v>
@@ -11023,7 +11057,7 @@
         <v>57</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>14</v>
@@ -11065,7 +11099,7 @@
         <v>57</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F30" s="10" t="s">
         <v>14</v>
@@ -11107,7 +11141,7 @@
         <v>57</v>
       </c>
       <c r="E31" s="15" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="F31" s="16" t="s">
         <v>14</v>
@@ -11275,7 +11309,7 @@
         <v>52</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J36" s="10">
         <f>H3</f>
@@ -11297,7 +11331,7 @@
         <v>3</v>
       </c>
       <c r="O36" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="P36" s="10">
         <f t="shared" ref="P36:P42" si="4">O36-I36</f>
@@ -11338,7 +11372,7 @@
         <v>52</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J37" s="10">
         <f>H3</f>
@@ -11360,7 +11394,7 @@
         <v>3</v>
       </c>
       <c r="O37" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="P37" s="10">
         <f t="shared" si="4"/>
@@ -11401,7 +11435,7 @@
         <v>52</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J38" s="10">
         <f>H3</f>
@@ -11423,7 +11457,7 @@
         <v>3</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="P38" s="10">
         <f t="shared" si="4"/>
@@ -11464,7 +11498,7 @@
         <v>52</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J39" s="10">
         <f>H3</f>
@@ -11486,7 +11520,7 @@
         <v>3</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="P39" s="10">
         <f t="shared" si="4"/>
@@ -11527,7 +11561,7 @@
         <v>52</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J40" s="10">
         <f>H3</f>
@@ -11549,7 +11583,7 @@
         <v>3</v>
       </c>
       <c r="O40" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="P40" s="10">
         <f t="shared" si="4"/>
@@ -11590,7 +11624,7 @@
         <v>52</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J41" s="10">
         <f>H3</f>
@@ -11612,7 +11646,7 @@
         <v>3</v>
       </c>
       <c r="O41" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="P41" s="10">
         <f t="shared" si="4"/>
@@ -11653,7 +11687,7 @@
         <v>52</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J42" s="10">
         <f>H3</f>
@@ -11675,7 +11709,7 @@
         <v>3</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="P42" s="10">
         <f t="shared" si="4"/>
@@ -11732,7 +11766,7 @@
     </row>
     <row r="44" spans="1:18">
       <c r="A44" s="23" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="B44" s="23"/>
       <c r="C44" s="23"/>
@@ -11814,7 +11848,7 @@
         <v>55</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="F46" s="10" t="s">
         <v>14</v>
@@ -11848,7 +11882,7 @@
         <v>3</v>
       </c>
       <c r="O46" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P46" s="10">
         <f t="shared" ref="P46:P52" si="9">O46-I46</f>
@@ -11877,7 +11911,7 @@
         <v>55</v>
       </c>
       <c r="E47" s="15" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="F47" s="10" t="s">
         <v>14</v>
@@ -11911,7 +11945,7 @@
         <v>3</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P47" s="10">
         <f t="shared" si="9"/>
@@ -11940,7 +11974,7 @@
         <v>55</v>
       </c>
       <c r="E48" s="15" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="F48" s="10" t="s">
         <v>14</v>
@@ -11974,7 +12008,7 @@
         <v>3</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P48" s="10">
         <f t="shared" si="9"/>
@@ -12003,7 +12037,7 @@
         <v>55</v>
       </c>
       <c r="E49" s="15" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="F49" s="10" t="s">
         <v>14</v>
@@ -12037,7 +12071,7 @@
         <v>3</v>
       </c>
       <c r="O49" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P49" s="10">
         <f t="shared" si="9"/>
@@ -12066,7 +12100,7 @@
         <v>55</v>
       </c>
       <c r="E50" s="15" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="F50" s="10" t="s">
         <v>14</v>
@@ -12100,7 +12134,7 @@
         <v>3</v>
       </c>
       <c r="O50" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P50" s="10">
         <f t="shared" si="9"/>
@@ -12129,7 +12163,7 @@
         <v>55</v>
       </c>
       <c r="E51" s="15" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="F51" s="10" t="s">
         <v>14</v>
@@ -12163,7 +12197,7 @@
         <v>3</v>
       </c>
       <c r="O51" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P51" s="10">
         <f t="shared" si="9"/>
@@ -12192,7 +12226,7 @@
         <v>55</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F52" s="10" t="s">
         <v>14</v>
@@ -12226,7 +12260,7 @@
         <v>3</v>
       </c>
       <c r="O52" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P52" s="10">
         <f t="shared" si="9"/>
@@ -12255,7 +12289,7 @@
         <v>57</v>
       </c>
       <c r="E53" s="15" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="F53" s="10" t="s">
         <v>14</v>
@@ -12289,7 +12323,7 @@
         <v>3</v>
       </c>
       <c r="O53" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P53" s="10">
         <f t="shared" ref="P53:P59" si="14">O53-I53</f>
@@ -12318,7 +12352,7 @@
         <v>57</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="F54" s="10" t="s">
         <v>14</v>
@@ -12352,7 +12386,7 @@
         <v>3</v>
       </c>
       <c r="O54" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P54" s="10">
         <f t="shared" si="14"/>
@@ -12381,7 +12415,7 @@
         <v>57</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>14</v>
@@ -12415,7 +12449,7 @@
         <v>3</v>
       </c>
       <c r="O55" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P55" s="10">
         <f t="shared" si="14"/>
@@ -12444,7 +12478,7 @@
         <v>57</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="F56" s="10" t="s">
         <v>14</v>
@@ -12478,7 +12512,7 @@
         <v>3</v>
       </c>
       <c r="O56" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P56" s="10">
         <f t="shared" si="14"/>
@@ -12507,7 +12541,7 @@
         <v>57</v>
       </c>
       <c r="E57" s="15" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>14</v>
@@ -12541,7 +12575,7 @@
         <v>3</v>
       </c>
       <c r="O57" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P57" s="10">
         <f t="shared" si="14"/>
@@ -12570,7 +12604,7 @@
         <v>57</v>
       </c>
       <c r="E58" s="15" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F58" s="10" t="s">
         <v>14</v>
@@ -12604,7 +12638,7 @@
         <v>3</v>
       </c>
       <c r="O58" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P58" s="10">
         <f t="shared" si="14"/>
@@ -12633,7 +12667,7 @@
         <v>57</v>
       </c>
       <c r="E59" s="15" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>14</v>
@@ -12667,7 +12701,7 @@
         <v>3</v>
       </c>
       <c r="O59" s="1" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="P59" s="10">
         <f t="shared" si="14"/>
@@ -12869,23 +12903,23 @@
   <dimension ref="A1:XEQ63"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="12.1428571428571" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.8190476190476" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.2761904761905" style="1" customWidth="1"/>
-    <col min="4" max="5" width="34.4571428571429" style="1" customWidth="1"/>
-    <col min="6" max="9" width="34.2761904761905" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15.3619047619048" style="1" customWidth="1"/>
-    <col min="11" max="11" width="34.2761904761905" style="1" customWidth="1"/>
-    <col min="12" max="12" width="14.3619047619048" style="1" customWidth="1"/>
-    <col min="13" max="13" width="16.1809523809524" style="1" customWidth="1"/>
-    <col min="14" max="14" width="19.3619047619048" style="1" customWidth="1"/>
-    <col min="15" max="15" width="19.6380952380952" style="1" customWidth="1"/>
-    <col min="16" max="16" width="15.9047619047619" style="1" customWidth="1"/>
-    <col min="17" max="17" width="21.1809523809524" style="1" customWidth="1"/>
-    <col min="18" max="18" width="16.2857142857143" style="1" customWidth="1"/>
-    <col min="19" max="21" width="19.6380952380952" style="1" customWidth="1"/>
-    <col min="22" max="16371" width="9.13333333333333" style="1"/>
-    <col min="16372" max="16384" width="9" style="2"/>
+    <col min="1" max="1" customWidth="true" style="1" width="12.1428571428571"/>
+    <col min="2" max="2" customWidth="true" style="1" width="11.8190476190476"/>
+    <col min="3" max="3" customWidth="true" style="1" width="17.2761904761905"/>
+    <col min="4" max="5" customWidth="true" style="1" width="34.4571428571429"/>
+    <col min="6" max="9" customWidth="true" style="1" width="34.2761904761905"/>
+    <col min="10" max="10" customWidth="true" style="1" width="15.3619047619048"/>
+    <col min="11" max="11" customWidth="true" style="1" width="34.2761904761905"/>
+    <col min="12" max="12" customWidth="true" style="1" width="14.3619047619048"/>
+    <col min="13" max="13" customWidth="true" style="1" width="16.1809523809524"/>
+    <col min="14" max="14" customWidth="true" style="1" width="19.3619047619048"/>
+    <col min="15" max="15" customWidth="true" style="1" width="19.6380952380952"/>
+    <col min="16" max="16" customWidth="true" style="1" width="15.9047619047619"/>
+    <col min="17" max="17" customWidth="true" style="1" width="21.1809523809524"/>
+    <col min="18" max="18" customWidth="true" style="1" width="16.2857142857143"/>
+    <col min="19" max="21" customWidth="true" style="1" width="19.6380952380952"/>
+    <col min="22" max="16371" style="1" width="9.13333333333333"/>
+    <col min="16372" max="16384" style="2" width="9.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33 16370:16371">
@@ -12962,7 +12996,7 @@
         <v>16</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>18</v>
@@ -12974,7 +13008,7 @@
         <v>3</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="J3" s="10">
         <f>I3+H3</f>
@@ -13310,10 +13344,10 @@
         <v>68</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J11" s="10">
         <f t="shared" ref="J11:J31" si="0">H11-I11</f>
@@ -13350,10 +13384,10 @@
         <v>68</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J12" s="10">
         <f t="shared" si="0"/>
@@ -13391,10 +13425,10 @@
         <v>68</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J13" s="10">
         <f t="shared" si="0"/>
@@ -13432,10 +13466,10 @@
         <v>68</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J14" s="10">
         <f t="shared" si="0"/>
@@ -13473,10 +13507,10 @@
         <v>68</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J15" s="10">
         <f t="shared" si="0"/>
@@ -13514,10 +13548,10 @@
         <v>68</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J16" s="10">
         <f t="shared" si="0"/>
@@ -13555,10 +13589,10 @@
         <v>68</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J17" s="10">
         <f t="shared" si="0"/>
@@ -13587,7 +13621,7 @@
         <v>55</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="F18" s="10" t="s">
         <v>14</v>
@@ -13600,7 +13634,7 @@
         <v>99771</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J18" s="10">
         <f t="shared" si="0"/>
@@ -13629,7 +13663,7 @@
         <v>55</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>14</v>
@@ -13642,7 +13676,7 @@
         <v>99771</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J19" s="10">
         <f t="shared" si="0"/>
@@ -13671,7 +13705,7 @@
         <v>55</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="F20" s="10" t="s">
         <v>14</v>
@@ -13684,7 +13718,7 @@
         <v>99771</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J20" s="10">
         <f t="shared" si="0"/>
@@ -13713,7 +13747,7 @@
         <v>55</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>14</v>
@@ -13726,7 +13760,7 @@
         <v>99771</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J21" s="10">
         <f t="shared" si="0"/>
@@ -13755,7 +13789,7 @@
         <v>55</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="F22" s="10" t="s">
         <v>14</v>
@@ -13768,7 +13802,7 @@
         <v>99771</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J22" s="10">
         <f t="shared" si="0"/>
@@ -13797,7 +13831,7 @@
         <v>55</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="F23" s="10" t="s">
         <v>14</v>
@@ -13810,7 +13844,7 @@
         <v>99771</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J23" s="10">
         <f t="shared" si="0"/>
@@ -13839,7 +13873,7 @@
         <v>55</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F24" s="10" t="s">
         <v>14</v>
@@ -13852,7 +13886,7 @@
         <v>99771</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J24" s="10">
         <f t="shared" si="0"/>
@@ -13881,7 +13915,7 @@
         <v>57</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>14</v>
@@ -13923,7 +13957,7 @@
         <v>57</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="F26" s="10" t="s">
         <v>14</v>
@@ -13965,7 +13999,7 @@
         <v>57</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>14</v>
@@ -14007,7 +14041,7 @@
         <v>57</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="F28" s="10" t="s">
         <v>14</v>
@@ -14049,7 +14083,7 @@
         <v>57</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>14</v>
@@ -14091,7 +14125,7 @@
         <v>57</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F30" s="10" t="s">
         <v>14</v>
@@ -14133,7 +14167,7 @@
         <v>57</v>
       </c>
       <c r="E31" s="15" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="F31" s="16" t="s">
         <v>14</v>
@@ -14303,7 +14337,7 @@
         <v>52</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J36" s="10">
         <f>H3</f>
@@ -14325,7 +14359,7 @@
         <v>3</v>
       </c>
       <c r="O36" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="P36" s="10">
         <f t="shared" ref="P36:P42" si="4">O36-I36</f>
@@ -14366,7 +14400,7 @@
         <v>52</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J37" s="10">
         <f>H3</f>
@@ -14388,7 +14422,7 @@
         <v>3</v>
       </c>
       <c r="O37" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="P37" s="10">
         <f t="shared" si="4"/>
@@ -14429,7 +14463,7 @@
         <v>52</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J38" s="10">
         <f>H3</f>
@@ -14451,7 +14485,7 @@
         <v>3</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="P38" s="10">
         <f t="shared" si="4"/>
@@ -14492,7 +14526,7 @@
         <v>52</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J39" s="10">
         <f>H3</f>
@@ -14514,7 +14548,7 @@
         <v>3</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="P39" s="10">
         <f t="shared" si="4"/>
@@ -14555,7 +14589,7 @@
         <v>52</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J40" s="10">
         <f>H3</f>
@@ -14577,7 +14611,7 @@
         <v>3</v>
       </c>
       <c r="O40" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="P40" s="10">
         <f t="shared" si="4"/>
@@ -14618,7 +14652,7 @@
         <v>52</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J41" s="10">
         <f>H3</f>
@@ -14640,7 +14674,7 @@
         <v>3</v>
       </c>
       <c r="O41" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="P41" s="10">
         <f t="shared" si="4"/>
@@ -14681,7 +14715,7 @@
         <v>52</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J42" s="10">
         <f>H3</f>
@@ -14703,7 +14737,7 @@
         <v>3</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="P42" s="10">
         <f t="shared" si="4"/>
@@ -14732,7 +14766,7 @@
         <v>55</v>
       </c>
       <c r="E43" s="15" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>14</v>
@@ -14795,7 +14829,7 @@
         <v>55</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="F44" s="10" t="s">
         <v>14</v>
@@ -14858,7 +14892,7 @@
         <v>55</v>
       </c>
       <c r="E45" s="15" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>14</v>
@@ -14921,7 +14955,7 @@
         <v>55</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="F46" s="10" t="s">
         <v>14</v>
@@ -14984,7 +15018,7 @@
         <v>55</v>
       </c>
       <c r="E47" s="15" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="F47" s="10" t="s">
         <v>14</v>
@@ -15047,7 +15081,7 @@
         <v>55</v>
       </c>
       <c r="E48" s="15" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="F48" s="10" t="s">
         <v>14</v>
@@ -15110,7 +15144,7 @@
         <v>55</v>
       </c>
       <c r="E49" s="15" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F49" s="10" t="s">
         <v>14</v>
@@ -15173,7 +15207,7 @@
         <v>57</v>
       </c>
       <c r="E50" s="15" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="F50" s="10" t="s">
         <v>14</v>
@@ -15236,7 +15270,7 @@
         <v>57</v>
       </c>
       <c r="E51" s="15" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="F51" s="10" t="s">
         <v>14</v>
@@ -15299,7 +15333,7 @@
         <v>57</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="F52" s="10" t="s">
         <v>14</v>
@@ -15362,7 +15396,7 @@
         <v>57</v>
       </c>
       <c r="E53" s="15" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="F53" s="10" t="s">
         <v>14</v>
@@ -15425,7 +15459,7 @@
         <v>57</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="F54" s="10" t="s">
         <v>14</v>
@@ -15488,7 +15522,7 @@
         <v>57</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>14</v>
@@ -15551,7 +15585,7 @@
         <v>57</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="F56" s="10" t="s">
         <v>14</v>

</xml_diff>